<commit_message>
DOC-002-R2: cobertura temporal de la financiación (brecha del año 0 contra fuentes con desembolso efectivo, tesorería proyectada y déficits por período), inventario trazable de salidas de caja del año 0 con barrido y devengado/pagado distinguidos, y escudo fiscal clasificado con contrafactual transitivo y hallazgo explícito cuando no puede calcularse
</commit_message>
<xml_diff>
--- a/docs/ejemplos/Ejemplo_Clinica_Libro_con_formulas.xlsx
+++ b/docs/ejemplos/Ejemplo_Clinica_Libro_con_formulas.xlsx
@@ -58,7 +58,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <numFmts count="11">
+  <numFmts count="12">
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
@@ -68,8 +68,9 @@
     <numFmt numFmtId="171" formatCode="0.0"/>
     <numFmt numFmtId="172" formatCode="#,##0.0"/>
     <numFmt numFmtId="173" formatCode="0.0%"/>
-    <numFmt numFmtId="174" formatCode="0.0000"/>
-    <numFmt numFmtId="175" formatCode="0.0"/>
+    <numFmt numFmtId="174" formatCode="#,##0.0"/>
+    <numFmt numFmtId="175" formatCode="0.0000"/>
+    <numFmt numFmtId="176" formatCode="0.0"/>
   </numFmts>
   <fonts count="20" x14ac:knownFonts="1">
     <font>
@@ -381,7 +382,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -412,12 +413,13 @@
     <xf numFmtId="173" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="12" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="22" borderId="0" xfId="0" applyFill="1" applyNumberFormat="1"/>
-    <xf numFmtId="174" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1" applyNumberFormat="1"/>
+    <xf numFmtId="175" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="13" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="true"/>
     </xf>
-    <xf numFmtId="175" fontId="14" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="14" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="15" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="16" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -799,7 +801,7 @@
         <v>Fecha de exportación:</v>
       </c>
       <c r="B7" s="2" t="str">
-        <v>25/10/2026, 23:01:53</v>
+        <v>26/10/2026, 0:40:10</v>
       </c>
     </row>
     <row r="8">
@@ -940,7 +942,7 @@
       <c r="D4" s="19">
         <v>6</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="27">
         <v>96000</v>
       </c>
       <c r="F4" s="14">
@@ -965,7 +967,7 @@
       <c r="D5" s="19">
         <v>3</v>
       </c>
-      <c r="E5" s="26">
+      <c r="E5" s="27">
         <v>312000</v>
       </c>
       <c r="F5" s="14">
@@ -990,7 +992,7 @@
       <c r="D6" s="19">
         <v>12</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="27">
         <v>264000</v>
       </c>
       <c r="F6" s="14">
@@ -1015,7 +1017,7 @@
       <c r="D7" s="19">
         <v>6</v>
       </c>
-      <c r="E7" s="26">
+      <c r="E7" s="27">
         <v>168000</v>
       </c>
       <c r="F7" s="14">
@@ -1040,7 +1042,7 @@
       <c r="D8" s="19">
         <v>5</v>
       </c>
-      <c r="E8" s="26">
+      <c r="E8" s="27">
         <v>120000</v>
       </c>
       <c r="F8" s="14">
@@ -1065,7 +1067,7 @@
       <c r="D9" s="19">
         <v>1</v>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="27">
         <v>9600000</v>
       </c>
       <c r="F9" s="14">
@@ -1090,7 +1092,7 @@
       <c r="D10" s="19">
         <v>3</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="27">
         <v>312000</v>
       </c>
       <c r="F10" s="14">
@@ -1115,7 +1117,7 @@
       <c r="D11" s="19">
         <v>12</v>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="27">
         <v>264000</v>
       </c>
       <c r="F11" s="14">
@@ -1140,7 +1142,7 @@
       <c r="D12" s="19">
         <v>6</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="27">
         <v>168000</v>
       </c>
       <c r="F12" s="14">
@@ -1165,7 +1167,7 @@
       <c r="D13" s="19">
         <v>5</v>
       </c>
-      <c r="E13" s="26">
+      <c r="E13" s="27">
         <v>120000</v>
       </c>
       <c r="F13" s="14">
@@ -1190,7 +1192,7 @@
       <c r="D14" s="19">
         <v>1</v>
       </c>
-      <c r="E14" s="26">
+      <c r="E14" s="27">
         <v>9600000</v>
       </c>
       <c r="F14" s="14">
@@ -1215,7 +1217,7 @@
       <c r="D15" s="19">
         <v>3</v>
       </c>
-      <c r="E15" s="26">
+      <c r="E15" s="27">
         <v>312000</v>
       </c>
       <c r="F15" s="14">
@@ -1240,7 +1242,7 @@
       <c r="D16" s="19">
         <v>12</v>
       </c>
-      <c r="E16" s="26">
+      <c r="E16" s="27">
         <v>264000</v>
       </c>
       <c r="F16" s="14">
@@ -1265,7 +1267,7 @@
       <c r="D17" s="19">
         <v>6</v>
       </c>
-      <c r="E17" s="26">
+      <c r="E17" s="27">
         <v>168000</v>
       </c>
       <c r="F17" s="14">
@@ -1290,7 +1292,7 @@
       <c r="D18" s="19">
         <v>5</v>
       </c>
-      <c r="E18" s="26">
+      <c r="E18" s="27">
         <v>120000</v>
       </c>
       <c r="F18" s="14">
@@ -1315,7 +1317,7 @@
       <c r="D19" s="19">
         <v>1</v>
       </c>
-      <c r="E19" s="26">
+      <c r="E19" s="27">
         <v>9600000</v>
       </c>
       <c r="F19" s="14">
@@ -1340,7 +1342,7 @@
       <c r="D20" s="19">
         <v>3</v>
       </c>
-      <c r="E20" s="26">
+      <c r="E20" s="27">
         <v>312000</v>
       </c>
       <c r="F20" s="14">
@@ -1365,7 +1367,7 @@
       <c r="D21" s="19">
         <v>12</v>
       </c>
-      <c r="E21" s="26">
+      <c r="E21" s="27">
         <v>264000</v>
       </c>
       <c r="F21" s="14">
@@ -1390,7 +1392,7 @@
       <c r="D22" s="19">
         <v>6</v>
       </c>
-      <c r="E22" s="26">
+      <c r="E22" s="27">
         <v>168000</v>
       </c>
       <c r="F22" s="14">
@@ -1415,7 +1417,7 @@
       <c r="D23" s="19">
         <v>5</v>
       </c>
-      <c r="E23" s="26">
+      <c r="E23" s="27">
         <v>120000</v>
       </c>
       <c r="F23" s="14">
@@ -1440,7 +1442,7 @@
       <c r="D24" s="19">
         <v>1</v>
       </c>
-      <c r="E24" s="26">
+      <c r="E24" s="27">
         <v>9600000</v>
       </c>
       <c r="F24" s="14">
@@ -1465,7 +1467,7 @@
       <c r="D25" s="19">
         <v>3</v>
       </c>
-      <c r="E25" s="26">
+      <c r="E25" s="27">
         <v>312000</v>
       </c>
       <c r="F25" s="14">
@@ -1490,7 +1492,7 @@
       <c r="D26" s="19">
         <v>12</v>
       </c>
-      <c r="E26" s="26">
+      <c r="E26" s="27">
         <v>264000</v>
       </c>
       <c r="F26" s="14">
@@ -1515,7 +1517,7 @@
       <c r="D27" s="19">
         <v>6</v>
       </c>
-      <c r="E27" s="26">
+      <c r="E27" s="27">
         <v>168000</v>
       </c>
       <c r="F27" s="14">
@@ -1540,7 +1542,7 @@
       <c r="D28" s="19">
         <v>5</v>
       </c>
-      <c r="E28" s="26">
+      <c r="E28" s="27">
         <v>120000</v>
       </c>
       <c r="F28" s="14">
@@ -1565,7 +1567,7 @@
       <c r="D29" s="19">
         <v>1</v>
       </c>
-      <c r="E29" s="26">
+      <c r="E29" s="27">
         <v>9600000</v>
       </c>
       <c r="F29" s="14">
@@ -1590,7 +1592,7 @@
       <c r="D30" s="19">
         <v>3</v>
       </c>
-      <c r="E30" s="26">
+      <c r="E30" s="27">
         <v>312000</v>
       </c>
       <c r="F30" s="14">
@@ -1615,7 +1617,7 @@
       <c r="D31" s="19">
         <v>12</v>
       </c>
-      <c r="E31" s="26">
+      <c r="E31" s="27">
         <v>264000</v>
       </c>
       <c r="F31" s="14">
@@ -1640,7 +1642,7 @@
       <c r="D32" s="19">
         <v>6</v>
       </c>
-      <c r="E32" s="26">
+      <c r="E32" s="27">
         <v>168000</v>
       </c>
       <c r="F32" s="14">
@@ -1665,7 +1667,7 @@
       <c r="D33" s="19">
         <v>5</v>
       </c>
-      <c r="E33" s="26">
+      <c r="E33" s="27">
         <v>120000</v>
       </c>
       <c r="F33" s="14">
@@ -1690,7 +1692,7 @@
       <c r="D34" s="19">
         <v>1</v>
       </c>
-      <c r="E34" s="26">
+      <c r="E34" s="27">
         <v>9600000</v>
       </c>
       <c r="F34" s="14">
@@ -1715,7 +1717,7 @@
       <c r="D35" s="19">
         <v>3</v>
       </c>
-      <c r="E35" s="26">
+      <c r="E35" s="27">
         <v>312000</v>
       </c>
       <c r="F35" s="14">
@@ -1740,7 +1742,7 @@
       <c r="D36" s="19">
         <v>12</v>
       </c>
-      <c r="E36" s="26">
+      <c r="E36" s="27">
         <v>264000</v>
       </c>
       <c r="F36" s="14">
@@ -1765,7 +1767,7 @@
       <c r="D37" s="19">
         <v>6</v>
       </c>
-      <c r="E37" s="26">
+      <c r="E37" s="27">
         <v>168000</v>
       </c>
       <c r="F37" s="14">
@@ -1790,7 +1792,7 @@
       <c r="D38" s="19">
         <v>5</v>
       </c>
-      <c r="E38" s="26">
+      <c r="E38" s="27">
         <v>120000</v>
       </c>
       <c r="F38" s="14">
@@ -1815,7 +1817,7 @@
       <c r="D39" s="19">
         <v>1</v>
       </c>
-      <c r="E39" s="26">
+      <c r="E39" s="27">
         <v>9600000</v>
       </c>
       <c r="F39" s="14">
@@ -1840,7 +1842,7 @@
       <c r="D40" s="19">
         <v>3</v>
       </c>
-      <c r="E40" s="26">
+      <c r="E40" s="27">
         <v>312000</v>
       </c>
       <c r="F40" s="14">
@@ -1865,7 +1867,7 @@
       <c r="D41" s="19">
         <v>12</v>
       </c>
-      <c r="E41" s="26">
+      <c r="E41" s="27">
         <v>264000</v>
       </c>
       <c r="F41" s="14">
@@ -1890,7 +1892,7 @@
       <c r="D42" s="19">
         <v>6</v>
       </c>
-      <c r="E42" s="26">
+      <c r="E42" s="27">
         <v>168000</v>
       </c>
       <c r="F42" s="14">
@@ -1915,7 +1917,7 @@
       <c r="D43" s="19">
         <v>5</v>
       </c>
-      <c r="E43" s="26">
+      <c r="E43" s="27">
         <v>120000</v>
       </c>
       <c r="F43" s="14">
@@ -1940,7 +1942,7 @@
       <c r="D44" s="19">
         <v>1</v>
       </c>
-      <c r="E44" s="26">
+      <c r="E44" s="27">
         <v>9600000</v>
       </c>
       <c r="F44" s="14">
@@ -1965,7 +1967,7 @@
       <c r="D45" s="19">
         <v>3</v>
       </c>
-      <c r="E45" s="26">
+      <c r="E45" s="27">
         <v>312000</v>
       </c>
       <c r="F45" s="14">
@@ -1990,7 +1992,7 @@
       <c r="D46" s="19">
         <v>12</v>
       </c>
-      <c r="E46" s="26">
+      <c r="E46" s="27">
         <v>264000</v>
       </c>
       <c r="F46" s="14">
@@ -2015,7 +2017,7 @@
       <c r="D47" s="19">
         <v>6</v>
       </c>
-      <c r="E47" s="26">
+      <c r="E47" s="27">
         <v>168000</v>
       </c>
       <c r="F47" s="14">
@@ -2040,7 +2042,7 @@
       <c r="D48" s="19">
         <v>5</v>
       </c>
-      <c r="E48" s="26">
+      <c r="E48" s="27">
         <v>120000</v>
       </c>
       <c r="F48" s="14">
@@ -2065,7 +2067,7 @@
       <c r="D49" s="19">
         <v>1</v>
       </c>
-      <c r="E49" s="26">
+      <c r="E49" s="27">
         <v>9600000</v>
       </c>
       <c r="F49" s="14">
@@ -2090,7 +2092,7 @@
       <c r="D50" s="19">
         <v>3</v>
       </c>
-      <c r="E50" s="26">
+      <c r="E50" s="27">
         <v>312000</v>
       </c>
       <c r="F50" s="14">
@@ -2115,7 +2117,7 @@
       <c r="D51" s="19">
         <v>12</v>
       </c>
-      <c r="E51" s="26">
+      <c r="E51" s="27">
         <v>264000</v>
       </c>
       <c r="F51" s="14">
@@ -2140,7 +2142,7 @@
       <c r="D52" s="19">
         <v>6</v>
       </c>
-      <c r="E52" s="26">
+      <c r="E52" s="27">
         <v>168000</v>
       </c>
       <c r="F52" s="14">
@@ -2165,7 +2167,7 @@
       <c r="D53" s="19">
         <v>5</v>
       </c>
-      <c r="E53" s="26">
+      <c r="E53" s="27">
         <v>120000</v>
       </c>
       <c r="F53" s="14">
@@ -2190,7 +2192,7 @@
       <c r="D54" s="19">
         <v>1</v>
       </c>
-      <c r="E54" s="26">
+      <c r="E54" s="27">
         <v>9600000</v>
       </c>
       <c r="F54" s="14">
@@ -5004,10 +5006,10 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="26" t="str">
+      <c r="A97" s="27" t="str">
         <v>Gabinetes de atención (sillones)</v>
       </c>
-      <c r="B97" s="26" t="str">
+      <c r="B97" s="27" t="str">
         <v>gabinete</v>
       </c>
       <c r="C97" s="19">
@@ -5220,47 +5222,47 @@
       <c r="B105" s="2" t="str">
         <v>Gabinetes de atención (sillones) — escala pro-rata</v>
       </c>
-      <c r="J105" s="27">
+      <c r="J105" s="28">
         <f>=IF($J104&gt;$J103,$J103/$J104,1)</f>
         <v>1</v>
       </c>
-      <c r="K105" s="27">
+      <c r="K105" s="28">
         <f>=IF($K104&gt;$K103,$K103/$K104,1)</f>
         <v>1</v>
       </c>
-      <c r="L105" s="27">
+      <c r="L105" s="28">
         <f>=IF($L104&gt;$L103,$L103/$L104,1)</f>
         <v>1</v>
       </c>
-      <c r="M105" s="27">
+      <c r="M105" s="28">
         <f>=IF($M104&gt;$M103,$M103/$M104,1)</f>
         <v>1</v>
       </c>
-      <c r="N105" s="27">
+      <c r="N105" s="28">
         <f>=IF($N104&gt;$N103,$N103/$N104,1)</f>
         <v>1</v>
       </c>
-      <c r="O105" s="27">
+      <c r="O105" s="28">
         <f>=IF($O104&gt;$O103,$O103/$O104,1)</f>
         <v>1</v>
       </c>
-      <c r="P105" s="27">
+      <c r="P105" s="28">
         <f>=IF($P104&gt;$P103,$P103/$P104,1)</f>
         <v>1</v>
       </c>
-      <c r="Q105" s="27">
+      <c r="Q105" s="28">
         <f>=IF($Q104&gt;$Q103,$Q103/$Q104,1)</f>
         <v>1</v>
       </c>
-      <c r="R105" s="27">
+      <c r="R105" s="28">
         <f>=IF($R104&gt;$R103,$R103/$R104,1)</f>
         <v>1</v>
       </c>
-      <c r="S105" s="27">
+      <c r="S105" s="28">
         <f>=IF($S104&gt;$S103,$S103/$S104,1)</f>
         <v>1</v>
       </c>
-      <c r="T105" s="27">
+      <c r="T105" s="28">
         <f>=IF($T104&gt;$T103,$T103/$T104,1)</f>
         <v>1</v>
       </c>
@@ -5416,47 +5418,47 @@
       <c r="B109" s="2" t="str">
         <v>Equipos de imagenología dental — escala pro-rata</v>
       </c>
-      <c r="J109" s="27">
+      <c r="J109" s="28">
         <f>=IF($J108&gt;$J107,$J107/$J108,1)</f>
         <v>1</v>
       </c>
-      <c r="K109" s="27">
+      <c r="K109" s="28">
         <f>=IF($K108&gt;$K107,$K107/$K108,1)</f>
         <v>1</v>
       </c>
-      <c r="L109" s="27">
+      <c r="L109" s="28">
         <f>=IF($L108&gt;$L107,$L107/$L108,1)</f>
         <v>1</v>
       </c>
-      <c r="M109" s="27">
+      <c r="M109" s="28">
         <f>=IF($M108&gt;$M107,$M107/$M108,1)</f>
         <v>1</v>
       </c>
-      <c r="N109" s="27">
+      <c r="N109" s="28">
         <f>=IF($N108&gt;$N107,$N107/$N108,1)</f>
         <v>1</v>
       </c>
-      <c r="O109" s="27">
+      <c r="O109" s="28">
         <f>=IF($O108&gt;$O107,$O107/$O108,1)</f>
         <v>1</v>
       </c>
-      <c r="P109" s="27">
+      <c r="P109" s="28">
         <f>=IF($P108&gt;$P107,$P107/$P108,1)</f>
         <v>1</v>
       </c>
-      <c r="Q109" s="27">
+      <c r="Q109" s="28">
         <f>=IF($Q108&gt;$Q107,$Q107/$Q108,1)</f>
         <v>1</v>
       </c>
-      <c r="R109" s="27">
+      <c r="R109" s="28">
         <f>=IF($R108&gt;$R107,$R107/$R108,1)</f>
         <v>1</v>
       </c>
-      <c r="S109" s="27">
+      <c r="S109" s="28">
         <f>=IF($S108&gt;$S107,$S107/$S108,1)</f>
         <v>1</v>
       </c>
-      <c r="T109" s="27">
+      <c r="T109" s="28">
         <f>=IF($T108&gt;$T107,$T107/$T108,1)</f>
         <v>1</v>
       </c>
@@ -5612,47 +5614,47 @@
       <c r="B113" s="2" t="str">
         <v>Laboratorio de prótesis — escala pro-rata</v>
       </c>
-      <c r="J113" s="27">
+      <c r="J113" s="28">
         <f>=IF($J112&gt;$J111,$J111/$J112,1)</f>
         <v>1</v>
       </c>
-      <c r="K113" s="27">
+      <c r="K113" s="28">
         <f>=IF($K112&gt;$K111,$K111/$K112,1)</f>
         <v>1</v>
       </c>
-      <c r="L113" s="27">
+      <c r="L113" s="28">
         <f>=IF($L112&gt;$L111,$L111/$L112,1)</f>
         <v>1</v>
       </c>
-      <c r="M113" s="27">
+      <c r="M113" s="28">
         <f>=IF($M112&gt;$M111,$M111/$M112,1)</f>
         <v>1</v>
       </c>
-      <c r="N113" s="27">
+      <c r="N113" s="28">
         <f>=IF($N112&gt;$N111,$N111/$N112,1)</f>
         <v>1</v>
       </c>
-      <c r="O113" s="27">
+      <c r="O113" s="28">
         <f>=IF($O112&gt;$O111,$O111/$O112,1)</f>
         <v>1</v>
       </c>
-      <c r="P113" s="27">
+      <c r="P113" s="28">
         <f>=IF($P112&gt;$P111,$P111/$P112,1)</f>
         <v>1</v>
       </c>
-      <c r="Q113" s="27">
+      <c r="Q113" s="28">
         <f>=IF($Q112&gt;$Q111,$Q111/$Q112,1)</f>
         <v>1</v>
       </c>
-      <c r="R113" s="27">
+      <c r="R113" s="28">
         <f>=IF($R112&gt;$R111,$R111/$R112,1)</f>
         <v>1</v>
       </c>
-      <c r="S113" s="27">
+      <c r="S113" s="28">
         <f>=IF($S112&gt;$S111,$S111/$S112,1)</f>
         <v>1</v>
       </c>
-      <c r="T113" s="27">
+      <c r="T113" s="28">
         <f>=IF($T112&gt;$T111,$T111/$T112,1)</f>
         <v>1</v>
       </c>
@@ -5808,47 +5810,47 @@
       <c r="B117" s="2" t="str">
         <v>Profesionales estomatológicos — escala pro-rata</v>
       </c>
-      <c r="J117" s="27">
+      <c r="J117" s="28">
         <f>=IF($J116&gt;$J115,$J115/$J116,1)</f>
         <v>1</v>
       </c>
-      <c r="K117" s="27">
+      <c r="K117" s="28">
         <f>=IF($K116&gt;$K115,$K115/$K116,1)</f>
         <v>1</v>
       </c>
-      <c r="L117" s="27">
+      <c r="L117" s="28">
         <f>=IF($L116&gt;$L115,$L115/$L116,1)</f>
         <v>1</v>
       </c>
-      <c r="M117" s="27">
+      <c r="M117" s="28">
         <f>=IF($M116&gt;$M115,$M115/$M116,1)</f>
         <v>1</v>
       </c>
-      <c r="N117" s="27">
+      <c r="N117" s="28">
         <f>=IF($N116&gt;$N115,$N115/$N116,1)</f>
         <v>1</v>
       </c>
-      <c r="O117" s="27">
+      <c r="O117" s="28">
         <f>=IF($O116&gt;$O115,$O115/$O116,1)</f>
         <v>1</v>
       </c>
-      <c r="P117" s="27">
+      <c r="P117" s="28">
         <f>=IF($P116&gt;$P115,$P115/$P116,1)</f>
         <v>1</v>
       </c>
-      <c r="Q117" s="27">
+      <c r="Q117" s="28">
         <f>=IF($Q116&gt;$Q115,$Q115/$Q116,1)</f>
         <v>1</v>
       </c>
-      <c r="R117" s="27">
+      <c r="R117" s="28">
         <f>=IF($R116&gt;$R115,$R115/$R116,1)</f>
         <v>1</v>
       </c>
-      <c r="S117" s="27">
+      <c r="S117" s="28">
         <f>=IF($S116&gt;$S115,$S115/$S116,1)</f>
         <v>1</v>
       </c>
-      <c r="T117" s="27">
+      <c r="T117" s="28">
         <f>=IF($T116&gt;$T115,$T115/$T116,1)</f>
         <v>1</v>
       </c>
@@ -5996,40 +5998,40 @@
       <c r="B3" s="12" t="str">
         <v>Unidad</v>
       </c>
-      <c r="C3" s="28">
-        <v>0</v>
-      </c>
-      <c r="D3" s="28">
-        <v>1</v>
-      </c>
-      <c r="E3" s="28">
+      <c r="C3" s="29">
+        <v>0</v>
+      </c>
+      <c r="D3" s="29">
+        <v>1</v>
+      </c>
+      <c r="E3" s="29">
         <v>2</v>
       </c>
-      <c r="F3" s="28">
+      <c r="F3" s="29">
         <v>3</v>
       </c>
-      <c r="G3" s="28">
+      <c r="G3" s="29">
         <v>4</v>
       </c>
-      <c r="H3" s="28">
+      <c r="H3" s="29">
         <v>5</v>
       </c>
-      <c r="I3" s="28">
+      <c r="I3" s="29">
         <v>6</v>
       </c>
-      <c r="J3" s="28">
+      <c r="J3" s="29">
         <v>7</v>
       </c>
-      <c r="K3" s="28">
+      <c r="K3" s="29">
         <v>8</v>
       </c>
-      <c r="L3" s="28">
+      <c r="L3" s="29">
         <v>9</v>
       </c>
-      <c r="M3" s="28">
+      <c r="M3" s="29">
         <v>10</v>
       </c>
-      <c r="N3" s="28" t="str">
+      <c r="N3" s="29" t="str">
         <v>Total</v>
       </c>
     </row>
@@ -8006,40 +8008,40 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="str">
+      <c r="A3" s="29" t="str">
         <v>Concepto</v>
       </c>
-      <c r="B3" s="28">
-        <v>0</v>
-      </c>
-      <c r="C3" s="28">
-        <v>1</v>
-      </c>
-      <c r="D3" s="28">
+      <c r="B3" s="29">
+        <v>0</v>
+      </c>
+      <c r="C3" s="29">
+        <v>1</v>
+      </c>
+      <c r="D3" s="29">
         <v>2</v>
       </c>
-      <c r="E3" s="28">
+      <c r="E3" s="29">
         <v>3</v>
       </c>
-      <c r="F3" s="28">
+      <c r="F3" s="29">
         <v>4</v>
       </c>
-      <c r="G3" s="28">
+      <c r="G3" s="29">
         <v>5</v>
       </c>
-      <c r="H3" s="28">
+      <c r="H3" s="29">
         <v>6</v>
       </c>
-      <c r="I3" s="28">
+      <c r="I3" s="29">
         <v>7</v>
       </c>
-      <c r="J3" s="28">
+      <c r="J3" s="29">
         <v>8</v>
       </c>
-      <c r="K3" s="28">
+      <c r="K3" s="29">
         <v>9</v>
       </c>
-      <c r="L3" s="28">
+      <c r="L3" s="29">
         <v>10</v>
       </c>
     </row>
@@ -8431,7 +8433,7 @@
       <c r="A14" s="22" t="str">
         <v>PERÍODO DE RECUPERACIÓN — INVERSIÓN TOTAL (años)</v>
       </c>
-      <c r="B14" s="29">
+      <c r="B14" s="30">
         <f>=IF(COUNT(C11:L$11)=0,"No se recupera en el horizonte",MIN(C11:L$11))</f>
         <v>3.463532275371478</v>
       </c>
@@ -8440,7 +8442,7 @@
       <c r="A15" s="8" t="str">
         <v>Método: interpolación lineal (t−1) + |acumulado anterior| / (acumulado actual − acumulado anterior); el mínimo de los cruces detectados.</v>
       </c>
-      <c r="B15" s="29">
+      <c r="B15" s="30">
         <f>=IF(COUNT(C12:L$12)=0,"No se recupera en el horizonte",MIN(C12:L$12))</f>
         <v>3.216105035737436</v>
       </c>
@@ -8579,40 +8581,40 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="str">
+      <c r="A3" s="29" t="str">
         <v>Concepto</v>
       </c>
-      <c r="B3" s="28">
-        <v>0</v>
-      </c>
-      <c r="C3" s="28">
-        <v>1</v>
-      </c>
-      <c r="D3" s="28">
+      <c r="B3" s="29">
+        <v>0</v>
+      </c>
+      <c r="C3" s="29">
+        <v>1</v>
+      </c>
+      <c r="D3" s="29">
         <v>2</v>
       </c>
-      <c r="E3" s="28">
+      <c r="E3" s="29">
         <v>3</v>
       </c>
-      <c r="F3" s="28">
+      <c r="F3" s="29">
         <v>4</v>
       </c>
-      <c r="G3" s="28">
+      <c r="G3" s="29">
         <v>5</v>
       </c>
-      <c r="H3" s="28">
+      <c r="H3" s="29">
         <v>6</v>
       </c>
-      <c r="I3" s="28">
+      <c r="I3" s="29">
         <v>7</v>
       </c>
-      <c r="J3" s="28">
+      <c r="J3" s="29">
         <v>8</v>
       </c>
-      <c r="K3" s="28">
+      <c r="K3" s="29">
         <v>9</v>
       </c>
-      <c r="L3" s="28">
+      <c r="L3" s="29">
         <v>10</v>
       </c>
     </row>
@@ -9197,43 +9199,43 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="str">
+      <c r="A3" s="29" t="str">
         <v>Concepto</v>
       </c>
-      <c r="B3" s="28">
-        <v>0</v>
-      </c>
-      <c r="C3" s="28">
-        <v>1</v>
-      </c>
-      <c r="D3" s="28">
+      <c r="B3" s="29">
+        <v>0</v>
+      </c>
+      <c r="C3" s="29">
+        <v>1</v>
+      </c>
+      <c r="D3" s="29">
         <v>2</v>
       </c>
-      <c r="E3" s="28">
+      <c r="E3" s="29">
         <v>3</v>
       </c>
-      <c r="F3" s="28">
+      <c r="F3" s="29">
         <v>4</v>
       </c>
-      <c r="G3" s="28">
+      <c r="G3" s="29">
         <v>5</v>
       </c>
-      <c r="H3" s="28">
+      <c r="H3" s="29">
         <v>6</v>
       </c>
-      <c r="I3" s="28">
+      <c r="I3" s="29">
         <v>7</v>
       </c>
-      <c r="J3" s="28">
+      <c r="J3" s="29">
         <v>8</v>
       </c>
-      <c r="K3" s="28">
+      <c r="K3" s="29">
         <v>9</v>
       </c>
-      <c r="L3" s="28">
+      <c r="L3" s="29">
         <v>10</v>
       </c>
-      <c r="M3" s="28" t="str">
+      <c r="M3" s="29" t="str">
         <v>Total</v>
       </c>
     </row>
@@ -9745,13 +9747,13 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="str">
+      <c r="A3" s="29" t="str">
         <v>Categoría</v>
       </c>
-      <c r="B3" s="28" t="str">
+      <c r="B3" s="29" t="str">
         <v>Cantidad</v>
       </c>
-      <c r="C3" s="28" t="str">
+      <c r="C3" s="29" t="str">
         <v>Salario promedio anual (CUP)</v>
       </c>
     </row>
@@ -9807,7 +9809,7 @@
       <c r="A8" s="22" t="str">
         <v>Total (operación)</v>
       </c>
-      <c r="B8" s="30">
+      <c r="B8" s="31">
         <f>=SUM(B4:B7)</f>
         <v>27</v>
       </c>
@@ -9857,16 +9859,16 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="str">
+      <c r="A3" s="29" t="str">
         <v>Etapa</v>
       </c>
-      <c r="B3" s="28" t="str">
+      <c r="B3" s="29" t="str">
         <v>Inicio</v>
       </c>
-      <c r="C3" s="28" t="str">
+      <c r="C3" s="29" t="str">
         <v>Fin</v>
       </c>
-      <c r="D3" s="28" t="str">
+      <c r="D3" s="29" t="str">
         <v>Observación</v>
       </c>
     </row>
@@ -9992,19 +9994,19 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="str">
+      <c r="A3" s="29" t="str">
         <v>Concepto</v>
       </c>
-      <c r="B3" s="28" t="str">
+      <c r="B3" s="29" t="str">
         <v>Unidad</v>
       </c>
-      <c r="C3" s="28" t="str">
+      <c r="C3" s="29" t="str">
         <v>Cantidad</v>
       </c>
-      <c r="D3" s="28" t="str">
+      <c r="D3" s="29" t="str">
         <v>Período</v>
       </c>
-      <c r="E3" s="28" t="str">
+      <c r="E3" s="29" t="str">
         <v>Observación</v>
       </c>
     </row>
@@ -10199,7 +10201,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="str">
+      <c r="A3" s="29" t="str">
         <v>Caracterización de productos y servicios</v>
       </c>
       <c r="B3" s="2" t="str">
@@ -10207,7 +10209,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="str">
+      <c r="A4" s="29" t="str">
         <v>Requisitos regulatorios y registros</v>
       </c>
       <c r="B4" s="2" t="str">
@@ -10215,7 +10217,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="str">
+      <c r="A5" s="29" t="str">
         <v>Materias primas y materiales auxiliares</v>
       </c>
       <c r="B5" s="2" t="str">
@@ -10223,7 +10225,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="str">
+      <c r="A6" s="29" t="str">
         <v>Fuentes y ubicación de suministros</v>
       </c>
       <c r="B6" s="2" t="str">
@@ -10231,7 +10233,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="str">
+      <c r="A7" s="29" t="str">
         <v>Consumo estimado</v>
       </c>
       <c r="B7" s="2" t="str">
@@ -10239,7 +10241,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="str">
+      <c r="A8" s="29" t="str">
         <v>Demanda aparente</v>
       </c>
       <c r="B8" s="2" t="str">
@@ -10247,7 +10249,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="str">
+      <c r="A9" s="29" t="str">
         <v>Demanda solvente</v>
       </c>
       <c r="B9" s="2" t="str">
@@ -10255,7 +10257,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="str">
+      <c r="A10" s="29" t="str">
         <v>Método de estimación</v>
       </c>
       <c r="B10" s="2" t="str">
@@ -10263,7 +10265,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="str">
+      <c r="A11" s="29" t="str">
         <v>Fuentes consultadas (con fecha)</v>
       </c>
       <c r="B11" s="2" t="str">
@@ -10271,7 +10273,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="str">
+      <c r="A12" s="29" t="str">
         <v>Comercialización: exportaciones</v>
       </c>
       <c r="B12" s="2" t="str">
@@ -10279,7 +10281,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="str">
+      <c r="A13" s="29" t="str">
         <v>Comercialización: divisas</v>
       </c>
       <c r="B13" s="2" t="str">
@@ -10287,7 +10289,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="str">
+      <c r="A14" s="29" t="str">
         <v>Comercialización: moneda nacional</v>
       </c>
       <c r="B14" s="2" t="str">
@@ -10489,7 +10491,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="str">
+      <c r="A3" s="29" t="str">
         <v>Elaborado por</v>
       </c>
       <c r="B3" s="2" t="str">
@@ -10497,7 +10499,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="str">
+      <c r="A4" s="29" t="str">
         <v>Cargo</v>
       </c>
       <c r="B4" s="2" t="str">
@@ -10505,7 +10507,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="str">
+      <c r="A5" s="29" t="str">
         <v>Fecha</v>
       </c>
       <c r="B5" s="2" t="str">
@@ -10513,7 +10515,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="str">
+      <c r="A6" s="29" t="str">
         <v>Declaración de responsabilidad</v>
       </c>
       <c r="B6" s="2" t="str">
@@ -10521,7 +10523,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="str">
+      <c r="A7" s="29" t="str">
         <v>Nombre del proyecto</v>
       </c>
       <c r="B7" s="2" t="str">
@@ -10529,7 +10531,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="str">
+      <c r="A8" s="29" t="str">
         <v>Denominación de la propuesta</v>
       </c>
       <c r="B8" s="2" t="str">
@@ -10537,7 +10539,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="str">
+      <c r="A9" s="29" t="str">
         <v>Modalidad de inversión</v>
       </c>
       <c r="B9" s="2" t="str">
@@ -10545,7 +10547,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="str">
+      <c r="A10" s="29" t="str">
         <v>Objeto social o contractual</v>
       </c>
       <c r="B10" s="2" t="str">
@@ -10553,7 +10555,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="str">
+      <c r="A11" s="29" t="str">
         <v>Plazo de vigencia</v>
       </c>
       <c r="B11" s="2" t="str">
@@ -10561,7 +10563,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="str">
+      <c r="A12" s="29" t="str">
         <v>Fundamentación y propuesta de valor</v>
       </c>
       <c r="B12" s="2" t="str">
@@ -10569,7 +10571,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="str">
+      <c r="A13" s="29" t="str">
         <v>Relación con objetivos de la inversión extranjera</v>
       </c>
       <c r="B13" s="2" t="str">
@@ -10577,7 +10579,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="str">
+      <c r="A14" s="29" t="str">
         <v>Relación con el PNDES</v>
       </c>
       <c r="B14" s="2" t="str">
@@ -10585,7 +10587,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="str">
+      <c r="A15" s="29" t="str">
         <v>Relación con la estrategia territorial</v>
       </c>
       <c r="B15" s="2" t="str">
@@ -10593,7 +10595,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="str">
+      <c r="A16" s="29" t="str">
         <v>Bienes y servicios</v>
       </c>
       <c r="B16" s="2" t="str">
@@ -10601,7 +10603,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="str">
+      <c r="A17" s="29" t="str">
         <v>Mercado interno</v>
       </c>
       <c r="B17" s="2" t="str">
@@ -10609,7 +10611,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="28" t="str">
+      <c r="A18" s="29" t="str">
         <v>Mercado externo</v>
       </c>
       <c r="B18" s="2" t="str">
@@ -10617,7 +10619,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="str">
+      <c r="A19" s="29" t="str">
         <v>Regla de distribución de beneficios</v>
       </c>
       <c r="B19" s="2" t="str">
@@ -10625,7 +10627,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="28" t="str">
+      <c r="A20" s="29" t="str">
         <v>Inversionista extranjero — nombre</v>
       </c>
       <c r="B20" s="2" t="str">
@@ -10633,7 +10635,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="str">
+      <c r="A21" s="29" t="str">
         <v>Inversionista extranjero — domicilio</v>
       </c>
       <c r="B21" s="2" t="str">
@@ -10641,7 +10643,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="28" t="str">
+      <c r="A22" s="29" t="str">
         <v>Inversionista extranjero — identificación fiscal</v>
       </c>
       <c r="B22" s="2" t="str">
@@ -10649,7 +10651,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="str">
+      <c r="A23" s="29" t="str">
         <v>Inversionista extranjero — experiencia</v>
       </c>
       <c r="B23" s="2" t="str">
@@ -10657,7 +10659,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="28" t="str">
+      <c r="A24" s="29" t="str">
         <v>Inversionista extranjero — vinculación con Cuba</v>
       </c>
       <c r="B24" s="2" t="str">
@@ -10665,7 +10667,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="28" t="str">
+      <c r="A25" s="29" t="str">
         <v>Inversionista nacional — nombre</v>
       </c>
       <c r="B25" s="2" t="str">
@@ -10673,7 +10675,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="28" t="str">
+      <c r="A26" s="29" t="str">
         <v>Inversionista nacional — domicilio</v>
       </c>
       <c r="B26" s="2" t="str">
@@ -10681,7 +10683,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="str">
+      <c r="A27" s="29" t="str">
         <v>Inversionista nacional — identificación fiscal</v>
       </c>
       <c r="B27" s="2" t="str">
@@ -10689,7 +10691,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="str">
+      <c r="A28" s="29" t="str">
         <v>Inversionista nacional — experiencia</v>
       </c>
       <c r="B28" s="2" t="str">
@@ -10697,7 +10699,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="28" t="str">
+      <c r="A29" s="29" t="str">
         <v>Inversionista nacional — vinculación con Cuba</v>
       </c>
       <c r="B29" s="2" t="str">
@@ -10705,7 +10707,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="28" t="str">
+      <c r="A30" s="29" t="str">
         <v>Conclusiones (marco del usuario)</v>
       </c>
       <c r="B30" s="2" t="str">
@@ -10740,31 +10742,31 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="str">
+      <c r="A3" s="29" t="str">
         <v>ID</v>
       </c>
-      <c r="B3" s="28" t="str">
+      <c r="B3" s="29" t="str">
         <v>Nombre</v>
       </c>
-      <c r="C3" s="28" t="str">
+      <c r="C3" s="29" t="str">
         <v>Categoría</v>
       </c>
-      <c r="D3" s="28" t="str">
+      <c r="D3" s="29" t="str">
         <v>Ámbito</v>
       </c>
-      <c r="E3" s="28" t="str">
+      <c r="E3" s="29" t="str">
         <v>Unidad</v>
       </c>
-      <c r="F3" s="28" t="str">
+      <c r="F3" s="29" t="str">
         <v>Habilitada</v>
       </c>
-      <c r="G3" s="28" t="str">
+      <c r="G3" s="29" t="str">
         <v>Expresión activa (motor PLANEX)</v>
       </c>
-      <c r="H3" s="28" t="str">
+      <c r="H3" s="29" t="str">
         <v>Equivalente Excel (año 1)</v>
       </c>
-      <c r="I3" s="28" t="str">
+      <c r="I3" s="29" t="str">
         <v>Estado</v>
       </c>
     </row>
@@ -12290,7 +12292,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G35"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -12307,46 +12309,46 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="str">
+      <c r="A3" s="29" t="str">
         <v>Nivel</v>
       </c>
-      <c r="B3" s="28" t="str">
+      <c r="B3" s="29" t="str">
         <v>Código</v>
       </c>
-      <c r="C3" s="28" t="str">
+      <c r="C3" s="29" t="str">
         <v>Hallazgo</v>
       </c>
-      <c r="D3" s="28" t="str">
+      <c r="D3" s="29" t="str">
         <v>Partida</v>
       </c>
-      <c r="E3" s="28" t="str">
+      <c r="E3" s="29" t="str">
         <v>Consecuencia</v>
       </c>
-      <c r="F3" s="28" t="str">
+      <c r="F3" s="29" t="str">
         <v>Corrección</v>
       </c>
-      <c r="G3" s="28" t="str">
+      <c r="G3" s="29" t="str">
         <v>Afecta conclusiones</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="31" t="str">
+      <c r="A4" s="32" t="str">
         <v>advertencia_importante</v>
       </c>
       <c r="B4" s="2" t="str">
         <v>FINANCIACION_ANO0</v>
       </c>
       <c r="C4" s="2" t="str">
-        <v>Los gastos de la fase de montaje del año 0 — salidas de caja explícitas no capitalizables y NO incluidas en la inversión total (nómina de montaje 0,8: total 0,8 kUSD) — quedan SIN cobertura: las fuentes declaradas cubren la inversión total (1.480,0 kUSD), pero la necesidad total del arranque (inversión + salidas de caja netas del año 0 = 1.480,8 kUSD) excede la financiación disponible (1.480,0 kUSD) en 0,8 kUSD. Financie esa brecha (mayor capital de trabajo o aporte adicional) o declárela expresamente como supuesto pendiente. El gasto NO se deduce del resultado contable después de impuestos del año 0.</v>
+        <v>Los gastos de la fase de montaje del año 0 — salidas de caja explícitas no capitalizables y NO incluidas en la inversión total (nómina de montaje 0,8: total 0,8 kUSD) — quedan SIN cobertura temporal: la necesidad total del arranque (inversión 1.480,0 + salidas netas del año 0 = 1.480,8 kUSD) excede las fuentes con desembolso efectivo en el año 0 (1.480,0 kUSD) en 0,8 kUSD. La financiación comprometida total (1.480,0 kUSD) tampoco cubre la necesidad total (1.480,8 kUSD): brecha nominal de 0,8 kUSD. Financie esa brecha (mayor capital de trabajo, aporte anticipado o crédito con desembolso en el año 0) o declárela expresamente como supuesto pendiente. El gasto NO se deduce del resultado contable después de impuestos del año 0.</v>
       </c>
       <c r="D4" s="2" t="str">
         <v>financiero</v>
       </c>
       <c r="E4" s="2" t="str">
-        <v>La necesidad total de arranque (inversión más gastos del año 0) excede la financiación declarada: el plan presenta una brecha de caja no resuelta.</v>
+        <v>La necesidad total de arranque (inversión más salidas de caja del año 0) excede las fuentes con desembolso efectivo en el año 0: el plan presenta una brecha de caja no resuelta cuando se produce.</v>
       </c>
       <c r="F4" s="2" t="str">
-        <v>Amplíe el capital de trabajo o las fuentes, o declare la brecha como supuesto pendiente de resolver.</v>
+        <v>Amplíe el capital de trabajo, antícipe aportes o el desembolso del crédito, o declare la brecha como supuesto pendiente de resolver.</v>
       </c>
       <c r="G4" s="2" t="str">
         <v>SÍ</v>
@@ -12492,22 +12494,22 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="str">
-        <v>informacion_pendiente</v>
+        <v>observacion_calidad</v>
       </c>
       <c r="B11" s="2" t="str">
-        <v>PENDIENTE</v>
+        <v>SUPUESTO_IMPUESTO_MISMO_PERIODO</v>
       </c>
       <c r="C11" s="2" t="str">
-        <v>Falta identificar al elaborador del plan (4.1): el campo está vacío o marcado como pendiente.</v>
+        <v>El impuesto sobre utilidades del modelo es un DEVENGADO contable (regla editable): el modelo simplificado SUPONE que se paga dentro del mismo período, sin calendario tributario. Ese supuesto se distingue expresamente de un pago verificado: con un calendario de pagos real (fracciones, diferimientos, pago al año siguiente) la tesorería proyectada y la necesidad de caja del arranque cambiarían.</v>
       </c>
       <c r="D11" s="2" t="str">
-        <v>4.1</v>
+        <v>impuesto_utilidades_k</v>
       </c>
       <c r="E11" s="2" t="str">
-        <v>El apartado no está completado sustantivamente.</v>
+        <v>La tesorería proyectada descansa en un supuesto de pago simultáneo, no en un calendario tributario verificado.</v>
       </c>
       <c r="F11" s="2" t="str">
-        <v>Complete la información o declare expresamente que está pendiente.</v>
+        <v>Documente la regla de pago tributaria aplicable (fuente y fecha) o modele el calendario de pagos si difiere del mismo período.</v>
       </c>
       <c r="G11" s="2" t="str">
         <v>No</v>
@@ -12515,22 +12517,22 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="str">
-        <v>informacion_pendiente</v>
+        <v>observacion_calidad</v>
       </c>
       <c r="B12" s="2" t="str">
-        <v>PENDIENTE</v>
+        <v>ESCUDO_FISCAL_CLASE</v>
       </c>
       <c r="C12" s="2" t="str">
-        <v>Falta la firma o identificación del elaborador (4.1).</v>
+        <v>Escudo fiscal — clasificación de la regla de impuestos activa: base directa. La regla de impuestos grava directamente la utilidad antes de intereses (referencia directa a «utilidad_antes_impuestos_k»): el escudo se calcula reevaluando la MISMA regla con la base hipotética sin intereses, respetando topes, mínimos y condiciones de su fórmula.</v>
       </c>
       <c r="D12" s="2" t="str">
-        <v>4.1</v>
+        <v>escudo fiscal</v>
       </c>
       <c r="E12" s="2" t="str">
-        <v>El apartado no está completado sustantivamente.</v>
+        <v>Clasificación documentada: la valoración de los flujos conoce qué reevalúa y qué no.</v>
       </c>
       <c r="F12" s="2" t="str">
-        <v>Complete la información o declare expresamente que está pendiente.</v>
+        <v>Mantenga la regla de impuestos reevaluable (sin dependencias circulares ni errores de dominio con la base hipotética).</v>
       </c>
       <c r="G12" s="2" t="str">
         <v>No</v>
@@ -12544,7 +12546,7 @@
         <v>PENDIENTE</v>
       </c>
       <c r="C13" s="2" t="str">
-        <v>La declaración de responsabilidad no ha sido aceptada (4.1): el documento NO está en condiciones de presentarse como definitivo.</v>
+        <v>Falta identificar al elaborador del plan (4.1): el campo está vacío o marcado como pendiente.</v>
       </c>
       <c r="D13" s="2" t="str">
         <v>4.1</v>
@@ -12564,166 +12566,212 @@
         <v>informacion_pendiente</v>
       </c>
       <c r="B14" s="2" t="str">
-        <v>REFERENCIA_HIPOTESIS</v>
+        <v>PENDIENTE</v>
       </c>
       <c r="C14" s="2" t="str">
-        <v>5 aportación(es) declaran una «referencia documental» que en realidad es una HIPÓTESIS de demostración (figuran como ficticia, ilustrativa, proforma o pendiente). Una referencia documental exigible debe identificar el documento, su emisor y su fecha, y adjuntar el soporte cuando corresponda.</v>
+        <v>Falta la firma o identificación del elaborador (4.1).</v>
       </c>
       <c r="D14" s="2" t="str">
-        <v>aportaciones</v>
+        <v>4.1</v>
       </c>
       <c r="E14" s="2" t="str">
-        <v>Los aportes no cuentan con respaldo acreditado: el plan no está en condiciones de presentarse oficialmente.</v>
+        <v>El apartado no está completado sustantivamente.</v>
       </c>
       <c r="F14" s="2" t="str">
-        <v>Sustituya las referencias hipotéticas por documentos identificables (título, emisor, fecha) o declare la ausencia de soporte.</v>
+        <v>Complete la información o declare expresamente que está pendiente.</v>
       </c>
       <c r="G14" s="2" t="str">
         <v>No</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="str">
+        <v>informacion_pendiente</v>
+      </c>
+      <c r="B15" s="2" t="str">
+        <v>PENDIENTE</v>
+      </c>
+      <c r="C15" s="2" t="str">
+        <v>La declaración de responsabilidad no ha sido aceptada (4.1): el documento NO está en condiciones de presentarse como definitivo.</v>
+      </c>
+      <c r="D15" s="2" t="str">
+        <v>4.1</v>
+      </c>
+      <c r="E15" s="2" t="str">
+        <v>El apartado no está completado sustantivamente.</v>
+      </c>
+      <c r="F15" s="2" t="str">
+        <v>Complete la información o declare expresamente que está pendiente.</v>
+      </c>
+      <c r="G15" s="2" t="str">
+        <v>No</v>
+      </c>
+    </row>
     <row r="16">
-      <c r="A16" s="3" t="str">
+      <c r="A16" s="2" t="str">
+        <v>informacion_pendiente</v>
+      </c>
+      <c r="B16" s="2" t="str">
+        <v>REFERENCIA_HIPOTESIS</v>
+      </c>
+      <c r="C16" s="2" t="str">
+        <v>5 aportación(es) declaran una «referencia documental» que en realidad es una HIPÓTESIS de demostración (figuran como ficticia, ilustrativa, proforma o pendiente). Una referencia documental exigible debe identificar el documento, su emisor y su fecha, y adjuntar el soporte cuando corresponda.</v>
+      </c>
+      <c r="D16" s="2" t="str">
+        <v>aportaciones</v>
+      </c>
+      <c r="E16" s="2" t="str">
+        <v>Los aportes no cuentan con respaldo acreditado: el plan no está en condiciones de presentarse oficialmente.</v>
+      </c>
+      <c r="F16" s="2" t="str">
+        <v>Sustituya las referencias hipotéticas por documentos identificables (título, emisor, fecha) o declare la ausencia de soporte.</v>
+      </c>
+      <c r="G16" s="2" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="str">
         <v>RESUMEN DE CONTROL</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="28" t="str">
+    <row r="19">
+      <c r="A19" s="29" t="str">
         <v>Dimensión</v>
       </c>
-      <c r="B17" s="28" t="str">
+      <c r="B19" s="29" t="str">
         <v>Estado</v>
       </c>
-      <c r="C17" s="28" t="str">
+      <c r="C19" s="29" t="str">
         <v>Detalle</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="str">
-        <v>Integridad aritmética</v>
-      </c>
-      <c r="B18" s="32" t="str">
-        <v>ok</v>
-      </c>
-      <c r="C18" s="2" t="str">
-        <v>Las reglas evalúan sin errores, la deuda reconcilia saldo a saldo, la depreciación no excede las bases y FCFF/FCFE cumplen la identidad algebraica.</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="str">
-        <v>Coherencia financiera y contable</v>
-      </c>
-      <c r="B19" s="33" t="str">
-        <v>deficiente</v>
-      </c>
-      <c r="C19" s="2" t="str">
-        <v>Inversión 1.480,0 kUSD vs financiación disponible 1.480,0 kUSD (conciliación del desembolso inicial incluida en el informe); recuperación simple del proyecto 3,5 años; del capital aportado 3,2 años; capacidad verificada contra los recursos operativos.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="str">
-        <v>Evidencia y trazabilidad de los supuestos</v>
-      </c>
-      <c r="B20" s="34" t="str">
-        <v>deficiente</v>
+        <v>Integridad aritmética</v>
+      </c>
+      <c r="B20" s="33" t="str">
+        <v>ok</v>
       </c>
       <c r="C20" s="2" t="str">
-        <v>4 parámetro(s) de demostración sin validación normativa; 5 aportación(es) sin referencia documental IDENTIFICABLE (vacía o hipótesis); 0 con referencia declarada. Las referencias hipotéticas NO cuentan como fuentes validadas.</v>
+        <v>Las reglas evalúan sin errores, la deuda reconcilia saldo a saldo, la depreciación no excede las bases y FCFF/FCFE cumplen la identidad algebraica.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="str">
-        <v>Cumplimiento de la estructura metodológica</v>
+        <v>Coherencia financiera y contable</v>
       </c>
       <c r="B21" s="34" t="str">
         <v>deficiente</v>
       </c>
       <c r="C21" s="2" t="str">
-        <v>Apartados 4.1–4.12 con 4 elemento(s) pendiente(s). Pendientes: 4.1, aportaciones. La completitud formal no equivale a validación de contenido.</v>
+        <v>Inversión 1.480,0 kUSD vs financiación comprometida 1.480,0 kUSD (conciliación total) y fuentes con desembolso en el año 0 1.480,0 kUSD (conciliación temporal, incluida en el informe); recuperación simple del proyecto 3,5 años; del capital aportado 3,2 años; capacidad verificada contra los recursos operativos.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="str">
-        <v>Estado de validación normativa y comercial</v>
-      </c>
-      <c r="B22" s="31" t="str">
-        <v>aceptable</v>
+        <v>Evidencia y trazabilidad de los supuestos</v>
+      </c>
+      <c r="B22" s="35" t="str">
+        <v>deficiente</v>
       </c>
       <c r="C22" s="2" t="str">
-        <v>La aplicación NO valida el cumplimiento legal, tributario, sanitario ni de mercado: la estructura documental no equivale a validación normativa. Los requisitos regulatorios declarados están LISTADOS, no VERIFICADOS: cada autorización exige evidencia externa comprobable (número, emisor, fecha). La demanda solvente y los precios requieren fuentes con fecha.</v>
+        <v>4 parámetro(s) de demostración sin validación normativa; 5 aportación(es) sin referencia documental IDENTIFICABLE (vacía o hipótesis); 0 con referencia declarada. Las referencias hipotéticas NO cuentan como fuentes validadas.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="str">
+        <v>Cumplimiento de la estructura metodológica</v>
+      </c>
+      <c r="B23" s="35" t="str">
+        <v>deficiente</v>
+      </c>
+      <c r="C23" s="2" t="str">
+        <v>Apartados 4.1–4.12 con 4 elemento(s) pendiente(s). Pendientes: 4.1, aportaciones. La completitud formal no equivale a validación de contenido.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="str">
+        <v>Estado de validación normativa y comercial</v>
+      </c>
+      <c r="B24" s="32" t="str">
+        <v>aceptable</v>
+      </c>
+      <c r="C24" s="2" t="str">
+        <v>La aplicación NO valida el cumplimiento legal, tributario, sanitario ni de mercado: la estructura documental no equivale a validación normativa. Los requisitos regulatorios declarados están LISTADOS, no VERIFICADOS: cada autorización exige evidencia externa comprobable (número, emisor, fecha). La demanda solvente y los precios requieren fuentes con fecha.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="str">
         <v>Calidad documental</v>
       </c>
-      <c r="B23" s="31" t="str">
+      <c r="B25" s="32" t="str">
         <v>aceptable</v>
       </c>
-      <c r="C23" s="2" t="str">
+      <c r="C25" s="2" t="str">
         <v>Observaciones de calidad: 6; 0 análisis editados por revisar frente al modelo; campos obligatorios pendientes en 4.1: 3.</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="str">
-        <v>Conteo: 0 error(es) bloqueante(s), 1 advertencia(s) importante(s), 4 pendiente(s), 6 observación(es) de calidad.</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="str">
-        <v>ESTADO GENERAL DEL PLAN (DOC-002 §5): Borrador de demostración (datos ficticios). Plantilla de demostración con datos ficticios: sus cifras NO son datos reales y el informe no está en condiciones de presentarse a un cliente o inversionista.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="str">
+        <v>Conteo: 0 error(es) bloqueante(s), 1 advertencia(s) importante(s), 4 pendiente(s), 8 observación(es) de calidad.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="str">
+        <v>ESTADO GENERAL DEL PLAN (DOC-002 §5): Borrador de demostración (datos ficticios). Plantilla de demostración con datos ficticios: sus cifras NO son datos reales y el informe no está en condiciones de presentarse a un cliente o inversionista.</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="str">
         <v>La completitud formal de campos NO se usa como prueba de calidad: un apartado completo de supuestos sin respaldo sigue sin estar validado. Las seis dimensiones se evalúan de forma independiente.</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="str">
+    <row r="29">
+      <c r="A29" s="4" t="str">
         <v>Clasificación de hallazgos (misión §15)</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="str">
-        <v>error_bloqueante</v>
-      </c>
-      <c r="B28" s="8" t="str">
-        <v>El cálculo es inválido, una fórmula tiene referencias rotas o existe una inconsistencia que impide interpretar el resultado.</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="str">
-        <v>advertencia_importante</v>
-      </c>
-      <c r="B29" s="8" t="str">
-        <v>Capacidad insuficiente, financiación no garantizada, recuperación no alcanzada o supuestos críticos no validados.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="str">
-        <v>informacion_pendiente</v>
+        <v>error_bloqueante</v>
       </c>
       <c r="B30" s="8" t="str">
-        <v>Falta completar un campo, adjuntar evidencia o documentar un supuesto.</v>
+        <v>El cálculo es inválido, una fórmula tiene referencias rotas o existe una inconsistencia que impide interpretar el resultado.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="str">
+        <v>advertencia_importante</v>
+      </c>
+      <c r="B31" s="8" t="str">
+        <v>Capacidad insuficiente, financiación no garantizada, recuperación no alcanzada o supuestos críticos no validados.</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="str">
+        <v>informacion_pendiente</v>
+      </c>
+      <c r="B32" s="8" t="str">
+        <v>Falta completar un campo, adjuntar evidencia o documentar un supuesto.</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="str">
         <v>observacion_calidad</v>
       </c>
-      <c r="B31" s="8" t="str">
+      <c r="B33" s="8" t="str">
         <v>Recomendación de mejorar la redacción, la evidencia, el análisis o la presentación.</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="10" t="str">
+    <row r="35">
+      <c r="A35" s="10" t="str">
         <v>EJEMPLO ILUSTRATIVO CON DATOS FICTICIOS.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G35"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -15438,7 +15486,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:H36"/>
   <cols>
     <col min="1" max="1" width="48.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -15609,9 +15657,356 @@
         <v>Tasa, plazo, gracia, tipo de gracia y método de amortización: hoja Deuda (configuración editable) y hoja Parametros.</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="3" t="str">
+        <v>Cobertura temporal de la financiación y tesorería proyectada (por período)</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="str">
+        <v>Fuentes comprometidas para todo el proyecto: 1.480,0 kUSD. Disponibles con desembolso en el año 0: 1.480,0 kUSD. Brecha temporal del año 0: -0,8 kUSD (nominal: -0,8). Las «otras fuentes» no declaran fecha: se suponen del año 0.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="str">
+        <v>Período</v>
+      </c>
+      <c r="B22" s="12" t="str">
+        <v>Aportaciones del año</v>
+      </c>
+      <c r="C22" s="12" t="str">
+        <v>Otras fuentes</v>
+      </c>
+      <c r="D22" s="12" t="str">
+        <v>Crédito (desembolso)</v>
+      </c>
+      <c r="E22" s="12" t="str">
+        <v>Fuentes del período</v>
+      </c>
+      <c r="F22" s="12" t="str">
+        <v>Necesidades del período</v>
+      </c>
+      <c r="G22" s="12" t="str">
+        <v>Cobertura acumulada</v>
+      </c>
+      <c r="H22" s="12" t="str">
+        <v>Caja proyectada</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="str">
+        <v>Año 0 (montaje)</v>
+      </c>
+      <c r="B23" s="26">
+        <v>1180</v>
+      </c>
+      <c r="C23" s="26">
+        <v>0</v>
+      </c>
+      <c r="D23" s="26">
+        <v>300</v>
+      </c>
+      <c r="E23" s="6">
+        <f>=SUM(B23:D23)</f>
+        <v>1480</v>
+      </c>
+      <c r="F23" s="26">
+        <v>1480.7752355316286</v>
+      </c>
+      <c r="G23" s="26">
+        <v>-0.7752355316285957</v>
+      </c>
+      <c r="H23" s="26">
+        <v>-0.7752355316285957</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="str">
+        <v>Año 1</v>
+      </c>
+      <c r="B24" s="26">
+        <v>0</v>
+      </c>
+      <c r="C24" s="26">
+        <v>0</v>
+      </c>
+      <c r="D24" s="26">
+        <v>0</v>
+      </c>
+      <c r="E24" s="6">
+        <f>=SUM(B24:D24)</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="26">
+        <v>0</v>
+      </c>
+      <c r="G24" s="26">
+        <v>-0.7752355316285957</v>
+      </c>
+      <c r="H24" s="26">
+        <v>367.80659051144005</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="str">
+        <v>Año 2</v>
+      </c>
+      <c r="B25" s="26">
+        <v>0</v>
+      </c>
+      <c r="C25" s="26">
+        <v>0</v>
+      </c>
+      <c r="D25" s="26">
+        <v>0</v>
+      </c>
+      <c r="E25" s="6">
+        <f>=SUM(B25:D25)</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="26">
+        <v>0</v>
+      </c>
+      <c r="G25" s="26">
+        <v>-0.7752355316285957</v>
+      </c>
+      <c r="H25" s="26">
+        <v>709.1861541066621</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="str">
+        <v>Año 3</v>
+      </c>
+      <c r="B26" s="26">
+        <v>0</v>
+      </c>
+      <c r="C26" s="26">
+        <v>0</v>
+      </c>
+      <c r="D26" s="26">
+        <v>0</v>
+      </c>
+      <c r="E26" s="6">
+        <f>=SUM(B26:D26)</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="26">
+        <v>0</v>
+      </c>
+      <c r="G26" s="26">
+        <v>-0.7752355316285957</v>
+      </c>
+      <c r="H26" s="26">
+        <v>1089.0175671792701</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="str">
+        <v>Año 4</v>
+      </c>
+      <c r="B27" s="26">
+        <v>0</v>
+      </c>
+      <c r="C27" s="26">
+        <v>0</v>
+      </c>
+      <c r="D27" s="26">
+        <v>0</v>
+      </c>
+      <c r="E27" s="6">
+        <f>=SUM(B27:D27)</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="26">
+        <v>0</v>
+      </c>
+      <c r="G27" s="26">
+        <v>-0.7752355316285957</v>
+      </c>
+      <c r="H27" s="26">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="str">
+        <v>Año 5</v>
+      </c>
+      <c r="B28" s="26">
+        <v>0</v>
+      </c>
+      <c r="C28" s="26">
+        <v>0</v>
+      </c>
+      <c r="D28" s="26">
+        <v>0</v>
+      </c>
+      <c r="E28" s="6">
+        <f>=SUM(B28:D28)</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="26">
+        <v>0</v>
+      </c>
+      <c r="G28" s="26">
+        <v>-0.7752355316285957</v>
+      </c>
+      <c r="H28" s="26">
+        <v>1177.7743860151013</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="str">
+        <v>Año 6</v>
+      </c>
+      <c r="B29" s="26">
+        <v>0</v>
+      </c>
+      <c r="C29" s="26">
+        <v>0</v>
+      </c>
+      <c r="D29" s="26">
+        <v>0</v>
+      </c>
+      <c r="E29" s="6">
+        <f>=SUM(B29:D29)</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="26">
+        <v>0</v>
+      </c>
+      <c r="G29" s="26">
+        <v>-0.7752355316285957</v>
+      </c>
+      <c r="H29" s="26">
+        <v>1270.4924946498547</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="str">
+        <v>Año 7</v>
+      </c>
+      <c r="B30" s="26">
+        <v>0</v>
+      </c>
+      <c r="C30" s="26">
+        <v>0</v>
+      </c>
+      <c r="D30" s="26">
+        <v>0</v>
+      </c>
+      <c r="E30" s="6">
+        <f>=SUM(B30:D30)</f>
+        <v>0</v>
+      </c>
+      <c r="F30" s="26">
+        <v>150</v>
+      </c>
+      <c r="G30" s="26">
+        <v>-150.7752355316286</v>
+      </c>
+      <c r="H30" s="26">
+        <v>1333.2702859615779</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="str">
+        <v>Año 8</v>
+      </c>
+      <c r="B31" s="26">
+        <v>0</v>
+      </c>
+      <c r="C31" s="26">
+        <v>0</v>
+      </c>
+      <c r="D31" s="26">
+        <v>0</v>
+      </c>
+      <c r="E31" s="6">
+        <f>=SUM(B31:D31)</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="26">
+        <v>0</v>
+      </c>
+      <c r="G31" s="26">
+        <v>-150.7752355316286</v>
+      </c>
+      <c r="H31" s="26">
+        <v>1576.072512645714</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="str">
+        <v>Año 9</v>
+      </c>
+      <c r="B32" s="26">
+        <v>0</v>
+      </c>
+      <c r="C32" s="26">
+        <v>0</v>
+      </c>
+      <c r="D32" s="26">
+        <v>0</v>
+      </c>
+      <c r="E32" s="6">
+        <f>=SUM(B32:D32)</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="26">
+        <v>0</v>
+      </c>
+      <c r="G32" s="26">
+        <v>-150.7752355316286</v>
+      </c>
+      <c r="H32" s="26">
+        <v>1831.2342900295337</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="str">
+        <v>Año 10</v>
+      </c>
+      <c r="B33" s="26">
+        <v>0</v>
+      </c>
+      <c r="C33" s="26">
+        <v>0</v>
+      </c>
+      <c r="D33" s="26">
+        <v>0</v>
+      </c>
+      <c r="E33" s="6">
+        <f>=SUM(B33:D33)</f>
+        <v>0</v>
+      </c>
+      <c r="F33" s="26">
+        <v>0</v>
+      </c>
+      <c r="G33" s="26">
+        <v>-150.7752355316286</v>
+      </c>
+      <c r="H33" s="26">
+        <v>2101.862597535257</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="str">
+        <v>Control temporal:</v>
+      </c>
+      <c r="B35" s="25" t="str">
+        <f>=IF(MIN(H23:H33)&lt;-0.05,"DÉFICIT TEMPORAL","OK")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="str">
+        <v>Necesidades: año 0 = inversión total + salidas de caja no capitalizables del arranque (inventario: nómina de montaje + interés pagado + impuesto devengado − ingresos explícitos); años posteriores = CAPEX de ampliaciones. El impuesto se toma como devengado pagado en el mismo período (supuesto del modelo simplificado).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -15732,10 +16127,10 @@
       <c r="C4" s="16">
         <v>25</v>
       </c>
-      <c r="D4" s="26">
+      <c r="D4" s="27">
         <v>400</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="27">
         <v>0</v>
       </c>
       <c r="F4" s="16">
@@ -15810,10 +16205,10 @@
       <c r="C5" s="16">
         <v>35</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="27">
         <v>160</v>
       </c>
-      <c r="E5" s="26">
+      <c r="E5" s="27">
         <v>0</v>
       </c>
       <c r="F5" s="16">
@@ -15888,10 +16283,10 @@
       <c r="C6" s="16">
         <v>60</v>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="27">
         <v>220</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="27">
         <v>0</v>
       </c>
       <c r="F6" s="16">
@@ -15966,10 +16361,10 @@
       <c r="C7" s="16">
         <v>150</v>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="27">
         <v>70</v>
       </c>
-      <c r="E7" s="26">
+      <c r="E7" s="27">
         <v>0</v>
       </c>
       <c r="F7" s="16">
@@ -16044,10 +16439,10 @@
       <c r="C8" s="16">
         <v>120</v>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="27">
         <v>60</v>
       </c>
-      <c r="E8" s="26">
+      <c r="E8" s="27">
         <v>0</v>
       </c>
       <c r="F8" s="16">
@@ -16122,10 +16517,10 @@
       <c r="C9" s="16">
         <v>180</v>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="27">
         <v>35</v>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="27">
         <v>0</v>
       </c>
       <c r="F9" s="16">
@@ -16200,10 +16595,10 @@
       <c r="C10" s="16">
         <v>400</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="27">
         <v>28</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="27">
         <v>0</v>
       </c>
       <c r="F10" s="16">
@@ -16278,10 +16673,10 @@
       <c r="C11" s="16">
         <v>1200</v>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="27">
         <v>9</v>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="27">
         <v>0</v>
       </c>
       <c r="F11" s="16">
@@ -16356,10 +16751,10 @@
       <c r="C12" s="16">
         <v>45</v>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="27">
         <v>130</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="27">
         <v>0</v>
       </c>
       <c r="F12" s="16">
@@ -16434,10 +16829,10 @@
       <c r="C13" s="16">
         <v>25</v>
       </c>
-      <c r="D13" s="26">
+      <c r="D13" s="27">
         <v>400</v>
       </c>
-      <c r="E13" s="26">
+      <c r="E13" s="27">
         <v>0</v>
       </c>
       <c r="F13" s="16">
@@ -16512,10 +16907,10 @@
       <c r="C14" s="16">
         <v>35</v>
       </c>
-      <c r="D14" s="26">
+      <c r="D14" s="27">
         <v>160</v>
       </c>
-      <c r="E14" s="26">
+      <c r="E14" s="27">
         <v>0</v>
       </c>
       <c r="F14" s="16">
@@ -16590,10 +16985,10 @@
       <c r="C15" s="16">
         <v>60</v>
       </c>
-      <c r="D15" s="26">
+      <c r="D15" s="27">
         <v>220</v>
       </c>
-      <c r="E15" s="26">
+      <c r="E15" s="27">
         <v>0</v>
       </c>
       <c r="F15" s="16">
@@ -16668,10 +17063,10 @@
       <c r="C16" s="16">
         <v>150</v>
       </c>
-      <c r="D16" s="26">
+      <c r="D16" s="27">
         <v>70</v>
       </c>
-      <c r="E16" s="26">
+      <c r="E16" s="27">
         <v>0</v>
       </c>
       <c r="F16" s="16">
@@ -16746,10 +17141,10 @@
       <c r="C17" s="16">
         <v>120</v>
       </c>
-      <c r="D17" s="26">
+      <c r="D17" s="27">
         <v>60</v>
       </c>
-      <c r="E17" s="26">
+      <c r="E17" s="27">
         <v>0</v>
       </c>
       <c r="F17" s="16">
@@ -16824,10 +17219,10 @@
       <c r="C18" s="16">
         <v>180</v>
       </c>
-      <c r="D18" s="26">
+      <c r="D18" s="27">
         <v>35</v>
       </c>
-      <c r="E18" s="26">
+      <c r="E18" s="27">
         <v>0</v>
       </c>
       <c r="F18" s="16">
@@ -16902,10 +17297,10 @@
       <c r="C19" s="16">
         <v>400</v>
       </c>
-      <c r="D19" s="26">
+      <c r="D19" s="27">
         <v>28</v>
       </c>
-      <c r="E19" s="26">
+      <c r="E19" s="27">
         <v>0</v>
       </c>
       <c r="F19" s="16">
@@ -16980,10 +17375,10 @@
       <c r="C20" s="16">
         <v>1200</v>
       </c>
-      <c r="D20" s="26">
+      <c r="D20" s="27">
         <v>9</v>
       </c>
-      <c r="E20" s="26">
+      <c r="E20" s="27">
         <v>0</v>
       </c>
       <c r="F20" s="16">
@@ -17058,10 +17453,10 @@
       <c r="C21" s="16">
         <v>45</v>
       </c>
-      <c r="D21" s="26">
+      <c r="D21" s="27">
         <v>130</v>
       </c>
-      <c r="E21" s="26">
+      <c r="E21" s="27">
         <v>0</v>
       </c>
       <c r="F21" s="16">
@@ -17136,10 +17531,10 @@
       <c r="C22" s="16">
         <v>25</v>
       </c>
-      <c r="D22" s="26">
+      <c r="D22" s="27">
         <v>400</v>
       </c>
-      <c r="E22" s="26">
+      <c r="E22" s="27">
         <v>0</v>
       </c>
       <c r="F22" s="16">
@@ -17214,10 +17609,10 @@
       <c r="C23" s="16">
         <v>35</v>
       </c>
-      <c r="D23" s="26">
+      <c r="D23" s="27">
         <v>160</v>
       </c>
-      <c r="E23" s="26">
+      <c r="E23" s="27">
         <v>0</v>
       </c>
       <c r="F23" s="16">
@@ -17292,10 +17687,10 @@
       <c r="C24" s="16">
         <v>60</v>
       </c>
-      <c r="D24" s="26">
+      <c r="D24" s="27">
         <v>220</v>
       </c>
-      <c r="E24" s="26">
+      <c r="E24" s="27">
         <v>0</v>
       </c>
       <c r="F24" s="16">
@@ -17370,10 +17765,10 @@
       <c r="C25" s="16">
         <v>150</v>
       </c>
-      <c r="D25" s="26">
+      <c r="D25" s="27">
         <v>70</v>
       </c>
-      <c r="E25" s="26">
+      <c r="E25" s="27">
         <v>0</v>
       </c>
       <c r="F25" s="16">
@@ -17448,10 +17843,10 @@
       <c r="C26" s="16">
         <v>120</v>
       </c>
-      <c r="D26" s="26">
+      <c r="D26" s="27">
         <v>60</v>
       </c>
-      <c r="E26" s="26">
+      <c r="E26" s="27">
         <v>0</v>
       </c>
       <c r="F26" s="16">
@@ -17526,10 +17921,10 @@
       <c r="C27" s="16">
         <v>180</v>
       </c>
-      <c r="D27" s="26">
+      <c r="D27" s="27">
         <v>35</v>
       </c>
-      <c r="E27" s="26">
+      <c r="E27" s="27">
         <v>0</v>
       </c>
       <c r="F27" s="16">
@@ -17604,10 +17999,10 @@
       <c r="C28" s="16">
         <v>400</v>
       </c>
-      <c r="D28" s="26">
+      <c r="D28" s="27">
         <v>28</v>
       </c>
-      <c r="E28" s="26">
+      <c r="E28" s="27">
         <v>0</v>
       </c>
       <c r="F28" s="16">
@@ -17682,10 +18077,10 @@
       <c r="C29" s="16">
         <v>1200</v>
       </c>
-      <c r="D29" s="26">
+      <c r="D29" s="27">
         <v>9</v>
       </c>
-      <c r="E29" s="26">
+      <c r="E29" s="27">
         <v>0</v>
       </c>
       <c r="F29" s="16">
@@ -17760,10 +18155,10 @@
       <c r="C30" s="16">
         <v>45</v>
       </c>
-      <c r="D30" s="26">
+      <c r="D30" s="27">
         <v>130</v>
       </c>
-      <c r="E30" s="26">
+      <c r="E30" s="27">
         <v>0</v>
       </c>
       <c r="F30" s="16">
@@ -17838,10 +18233,10 @@
       <c r="C31" s="16">
         <v>25</v>
       </c>
-      <c r="D31" s="26">
+      <c r="D31" s="27">
         <v>400</v>
       </c>
-      <c r="E31" s="26">
+      <c r="E31" s="27">
         <v>0</v>
       </c>
       <c r="F31" s="16">
@@ -17916,10 +18311,10 @@
       <c r="C32" s="16">
         <v>35</v>
       </c>
-      <c r="D32" s="26">
+      <c r="D32" s="27">
         <v>160</v>
       </c>
-      <c r="E32" s="26">
+      <c r="E32" s="27">
         <v>0</v>
       </c>
       <c r="F32" s="16">
@@ -17994,10 +18389,10 @@
       <c r="C33" s="16">
         <v>60</v>
       </c>
-      <c r="D33" s="26">
+      <c r="D33" s="27">
         <v>220</v>
       </c>
-      <c r="E33" s="26">
+      <c r="E33" s="27">
         <v>0</v>
       </c>
       <c r="F33" s="16">
@@ -18072,10 +18467,10 @@
       <c r="C34" s="16">
         <v>150</v>
       </c>
-      <c r="D34" s="26">
+      <c r="D34" s="27">
         <v>70</v>
       </c>
-      <c r="E34" s="26">
+      <c r="E34" s="27">
         <v>0</v>
       </c>
       <c r="F34" s="16">
@@ -18150,10 +18545,10 @@
       <c r="C35" s="16">
         <v>120</v>
       </c>
-      <c r="D35" s="26">
+      <c r="D35" s="27">
         <v>60</v>
       </c>
-      <c r="E35" s="26">
+      <c r="E35" s="27">
         <v>0</v>
       </c>
       <c r="F35" s="16">
@@ -18228,10 +18623,10 @@
       <c r="C36" s="16">
         <v>180</v>
       </c>
-      <c r="D36" s="26">
+      <c r="D36" s="27">
         <v>35</v>
       </c>
-      <c r="E36" s="26">
+      <c r="E36" s="27">
         <v>0</v>
       </c>
       <c r="F36" s="16">
@@ -18306,10 +18701,10 @@
       <c r="C37" s="16">
         <v>400</v>
       </c>
-      <c r="D37" s="26">
+      <c r="D37" s="27">
         <v>28</v>
       </c>
-      <c r="E37" s="26">
+      <c r="E37" s="27">
         <v>0</v>
       </c>
       <c r="F37" s="16">
@@ -18384,10 +18779,10 @@
       <c r="C38" s="16">
         <v>1200</v>
       </c>
-      <c r="D38" s="26">
+      <c r="D38" s="27">
         <v>9</v>
       </c>
-      <c r="E38" s="26">
+      <c r="E38" s="27">
         <v>0</v>
       </c>
       <c r="F38" s="16">
@@ -18462,10 +18857,10 @@
       <c r="C39" s="16">
         <v>45</v>
       </c>
-      <c r="D39" s="26">
+      <c r="D39" s="27">
         <v>130</v>
       </c>
-      <c r="E39" s="26">
+      <c r="E39" s="27">
         <v>0</v>
       </c>
       <c r="F39" s="16">
@@ -18540,10 +18935,10 @@
       <c r="C40" s="16">
         <v>25</v>
       </c>
-      <c r="D40" s="26">
+      <c r="D40" s="27">
         <v>400</v>
       </c>
-      <c r="E40" s="26">
+      <c r="E40" s="27">
         <v>0</v>
       </c>
       <c r="F40" s="16">
@@ -18618,10 +19013,10 @@
       <c r="C41" s="16">
         <v>35</v>
       </c>
-      <c r="D41" s="26">
+      <c r="D41" s="27">
         <v>160</v>
       </c>
-      <c r="E41" s="26">
+      <c r="E41" s="27">
         <v>0</v>
       </c>
       <c r="F41" s="16">
@@ -18696,10 +19091,10 @@
       <c r="C42" s="16">
         <v>60</v>
       </c>
-      <c r="D42" s="26">
+      <c r="D42" s="27">
         <v>220</v>
       </c>
-      <c r="E42" s="26">
+      <c r="E42" s="27">
         <v>0</v>
       </c>
       <c r="F42" s="16">
@@ -18774,10 +19169,10 @@
       <c r="C43" s="16">
         <v>150</v>
       </c>
-      <c r="D43" s="26">
+      <c r="D43" s="27">
         <v>70</v>
       </c>
-      <c r="E43" s="26">
+      <c r="E43" s="27">
         <v>0</v>
       </c>
       <c r="F43" s="16">
@@ -18852,10 +19247,10 @@
       <c r="C44" s="16">
         <v>120</v>
       </c>
-      <c r="D44" s="26">
+      <c r="D44" s="27">
         <v>60</v>
       </c>
-      <c r="E44" s="26">
+      <c r="E44" s="27">
         <v>0</v>
       </c>
       <c r="F44" s="16">
@@ -18930,10 +19325,10 @@
       <c r="C45" s="16">
         <v>180</v>
       </c>
-      <c r="D45" s="26">
+      <c r="D45" s="27">
         <v>35</v>
       </c>
-      <c r="E45" s="26">
+      <c r="E45" s="27">
         <v>0</v>
       </c>
       <c r="F45" s="16">
@@ -19008,10 +19403,10 @@
       <c r="C46" s="16">
         <v>400</v>
       </c>
-      <c r="D46" s="26">
+      <c r="D46" s="27">
         <v>28</v>
       </c>
-      <c r="E46" s="26">
+      <c r="E46" s="27">
         <v>0</v>
       </c>
       <c r="F46" s="16">
@@ -19086,10 +19481,10 @@
       <c r="C47" s="16">
         <v>1200</v>
       </c>
-      <c r="D47" s="26">
+      <c r="D47" s="27">
         <v>9</v>
       </c>
-      <c r="E47" s="26">
+      <c r="E47" s="27">
         <v>0</v>
       </c>
       <c r="F47" s="16">
@@ -19164,10 +19559,10 @@
       <c r="C48" s="16">
         <v>45</v>
       </c>
-      <c r="D48" s="26">
+      <c r="D48" s="27">
         <v>130</v>
       </c>
-      <c r="E48" s="26">
+      <c r="E48" s="27">
         <v>0</v>
       </c>
       <c r="F48" s="16">
@@ -19242,10 +19637,10 @@
       <c r="C49" s="16">
         <v>25</v>
       </c>
-      <c r="D49" s="26">
+      <c r="D49" s="27">
         <v>400</v>
       </c>
-      <c r="E49" s="26">
+      <c r="E49" s="27">
         <v>0</v>
       </c>
       <c r="F49" s="16">
@@ -19320,10 +19715,10 @@
       <c r="C50" s="16">
         <v>35</v>
       </c>
-      <c r="D50" s="26">
+      <c r="D50" s="27">
         <v>160</v>
       </c>
-      <c r="E50" s="26">
+      <c r="E50" s="27">
         <v>0</v>
       </c>
       <c r="F50" s="16">
@@ -19398,10 +19793,10 @@
       <c r="C51" s="16">
         <v>60</v>
       </c>
-      <c r="D51" s="26">
+      <c r="D51" s="27">
         <v>220</v>
       </c>
-      <c r="E51" s="26">
+      <c r="E51" s="27">
         <v>0</v>
       </c>
       <c r="F51" s="16">
@@ -19476,10 +19871,10 @@
       <c r="C52" s="16">
         <v>150</v>
       </c>
-      <c r="D52" s="26">
+      <c r="D52" s="27">
         <v>70</v>
       </c>
-      <c r="E52" s="26">
+      <c r="E52" s="27">
         <v>0</v>
       </c>
       <c r="F52" s="16">
@@ -19554,10 +19949,10 @@
       <c r="C53" s="16">
         <v>120</v>
       </c>
-      <c r="D53" s="26">
+      <c r="D53" s="27">
         <v>60</v>
       </c>
-      <c r="E53" s="26">
+      <c r="E53" s="27">
         <v>0</v>
       </c>
       <c r="F53" s="16">
@@ -19632,10 +20027,10 @@
       <c r="C54" s="16">
         <v>180</v>
       </c>
-      <c r="D54" s="26">
+      <c r="D54" s="27">
         <v>35</v>
       </c>
-      <c r="E54" s="26">
+      <c r="E54" s="27">
         <v>0</v>
       </c>
       <c r="F54" s="16">
@@ -19710,10 +20105,10 @@
       <c r="C55" s="16">
         <v>400</v>
       </c>
-      <c r="D55" s="26">
+      <c r="D55" s="27">
         <v>28</v>
       </c>
-      <c r="E55" s="26">
+      <c r="E55" s="27">
         <v>0</v>
       </c>
       <c r="F55" s="16">
@@ -19788,10 +20183,10 @@
       <c r="C56" s="16">
         <v>1200</v>
       </c>
-      <c r="D56" s="26">
+      <c r="D56" s="27">
         <v>9</v>
       </c>
-      <c r="E56" s="26">
+      <c r="E56" s="27">
         <v>0</v>
       </c>
       <c r="F56" s="16">
@@ -19866,10 +20261,10 @@
       <c r="C57" s="16">
         <v>45</v>
       </c>
-      <c r="D57" s="26">
+      <c r="D57" s="27">
         <v>130</v>
       </c>
-      <c r="E57" s="26">
+      <c r="E57" s="27">
         <v>0</v>
       </c>
       <c r="F57" s="16">
@@ -19944,10 +20339,10 @@
       <c r="C58" s="16">
         <v>25</v>
       </c>
-      <c r="D58" s="26">
+      <c r="D58" s="27">
         <v>400</v>
       </c>
-      <c r="E58" s="26">
+      <c r="E58" s="27">
         <v>0</v>
       </c>
       <c r="F58" s="16">
@@ -20022,10 +20417,10 @@
       <c r="C59" s="16">
         <v>35</v>
       </c>
-      <c r="D59" s="26">
+      <c r="D59" s="27">
         <v>160</v>
       </c>
-      <c r="E59" s="26">
+      <c r="E59" s="27">
         <v>0</v>
       </c>
       <c r="F59" s="16">
@@ -20100,10 +20495,10 @@
       <c r="C60" s="16">
         <v>60</v>
       </c>
-      <c r="D60" s="26">
+      <c r="D60" s="27">
         <v>220</v>
       </c>
-      <c r="E60" s="26">
+      <c r="E60" s="27">
         <v>0</v>
       </c>
       <c r="F60" s="16">
@@ -20178,10 +20573,10 @@
       <c r="C61" s="16">
         <v>150</v>
       </c>
-      <c r="D61" s="26">
+      <c r="D61" s="27">
         <v>70</v>
       </c>
-      <c r="E61" s="26">
+      <c r="E61" s="27">
         <v>0</v>
       </c>
       <c r="F61" s="16">
@@ -20256,10 +20651,10 @@
       <c r="C62" s="16">
         <v>120</v>
       </c>
-      <c r="D62" s="26">
+      <c r="D62" s="27">
         <v>60</v>
       </c>
-      <c r="E62" s="26">
+      <c r="E62" s="27">
         <v>0</v>
       </c>
       <c r="F62" s="16">
@@ -20334,10 +20729,10 @@
       <c r="C63" s="16">
         <v>180</v>
       </c>
-      <c r="D63" s="26">
+      <c r="D63" s="27">
         <v>35</v>
       </c>
-      <c r="E63" s="26">
+      <c r="E63" s="27">
         <v>0</v>
       </c>
       <c r="F63" s="16">
@@ -20412,10 +20807,10 @@
       <c r="C64" s="16">
         <v>400</v>
       </c>
-      <c r="D64" s="26">
+      <c r="D64" s="27">
         <v>28</v>
       </c>
-      <c r="E64" s="26">
+      <c r="E64" s="27">
         <v>0</v>
       </c>
       <c r="F64" s="16">
@@ -20490,10 +20885,10 @@
       <c r="C65" s="16">
         <v>1200</v>
       </c>
-      <c r="D65" s="26">
+      <c r="D65" s="27">
         <v>9</v>
       </c>
-      <c r="E65" s="26">
+      <c r="E65" s="27">
         <v>0</v>
       </c>
       <c r="F65" s="16">
@@ -20568,10 +20963,10 @@
       <c r="C66" s="16">
         <v>45</v>
       </c>
-      <c r="D66" s="26">
+      <c r="D66" s="27">
         <v>130</v>
       </c>
-      <c r="E66" s="26">
+      <c r="E66" s="27">
         <v>0</v>
       </c>
       <c r="F66" s="16">
@@ -20646,10 +21041,10 @@
       <c r="C67" s="16">
         <v>25</v>
       </c>
-      <c r="D67" s="26">
+      <c r="D67" s="27">
         <v>400</v>
       </c>
-      <c r="E67" s="26">
+      <c r="E67" s="27">
         <v>0</v>
       </c>
       <c r="F67" s="16">
@@ -20724,10 +21119,10 @@
       <c r="C68" s="16">
         <v>35</v>
       </c>
-      <c r="D68" s="26">
+      <c r="D68" s="27">
         <v>160</v>
       </c>
-      <c r="E68" s="26">
+      <c r="E68" s="27">
         <v>0</v>
       </c>
       <c r="F68" s="16">
@@ -20802,10 +21197,10 @@
       <c r="C69" s="16">
         <v>60</v>
       </c>
-      <c r="D69" s="26">
+      <c r="D69" s="27">
         <v>220</v>
       </c>
-      <c r="E69" s="26">
+      <c r="E69" s="27">
         <v>0</v>
       </c>
       <c r="F69" s="16">
@@ -20880,10 +21275,10 @@
       <c r="C70" s="16">
         <v>150</v>
       </c>
-      <c r="D70" s="26">
+      <c r="D70" s="27">
         <v>70</v>
       </c>
-      <c r="E70" s="26">
+      <c r="E70" s="27">
         <v>0</v>
       </c>
       <c r="F70" s="16">
@@ -20958,10 +21353,10 @@
       <c r="C71" s="16">
         <v>120</v>
       </c>
-      <c r="D71" s="26">
+      <c r="D71" s="27">
         <v>60</v>
       </c>
-      <c r="E71" s="26">
+      <c r="E71" s="27">
         <v>0</v>
       </c>
       <c r="F71" s="16">
@@ -21036,10 +21431,10 @@
       <c r="C72" s="16">
         <v>180</v>
       </c>
-      <c r="D72" s="26">
+      <c r="D72" s="27">
         <v>35</v>
       </c>
-      <c r="E72" s="26">
+      <c r="E72" s="27">
         <v>0</v>
       </c>
       <c r="F72" s="16">
@@ -21114,10 +21509,10 @@
       <c r="C73" s="16">
         <v>400</v>
       </c>
-      <c r="D73" s="26">
+      <c r="D73" s="27">
         <v>28</v>
       </c>
-      <c r="E73" s="26">
+      <c r="E73" s="27">
         <v>0</v>
       </c>
       <c r="F73" s="16">
@@ -21192,10 +21587,10 @@
       <c r="C74" s="16">
         <v>1200</v>
       </c>
-      <c r="D74" s="26">
+      <c r="D74" s="27">
         <v>9</v>
       </c>
-      <c r="E74" s="26">
+      <c r="E74" s="27">
         <v>0</v>
       </c>
       <c r="F74" s="16">
@@ -21270,10 +21665,10 @@
       <c r="C75" s="16">
         <v>45</v>
       </c>
-      <c r="D75" s="26">
+      <c r="D75" s="27">
         <v>130</v>
       </c>
-      <c r="E75" s="26">
+      <c r="E75" s="27">
         <v>0</v>
       </c>
       <c r="F75" s="16">
@@ -21348,10 +21743,10 @@
       <c r="C76" s="16">
         <v>25</v>
       </c>
-      <c r="D76" s="26">
+      <c r="D76" s="27">
         <v>400</v>
       </c>
-      <c r="E76" s="26">
+      <c r="E76" s="27">
         <v>0</v>
       </c>
       <c r="F76" s="16">
@@ -21426,10 +21821,10 @@
       <c r="C77" s="16">
         <v>35</v>
       </c>
-      <c r="D77" s="26">
+      <c r="D77" s="27">
         <v>160</v>
       </c>
-      <c r="E77" s="26">
+      <c r="E77" s="27">
         <v>0</v>
       </c>
       <c r="F77" s="16">
@@ -21504,10 +21899,10 @@
       <c r="C78" s="16">
         <v>60</v>
       </c>
-      <c r="D78" s="26">
+      <c r="D78" s="27">
         <v>220</v>
       </c>
-      <c r="E78" s="26">
+      <c r="E78" s="27">
         <v>0</v>
       </c>
       <c r="F78" s="16">
@@ -21582,10 +21977,10 @@
       <c r="C79" s="16">
         <v>150</v>
       </c>
-      <c r="D79" s="26">
+      <c r="D79" s="27">
         <v>70</v>
       </c>
-      <c r="E79" s="26">
+      <c r="E79" s="27">
         <v>0</v>
       </c>
       <c r="F79" s="16">
@@ -21660,10 +22055,10 @@
       <c r="C80" s="16">
         <v>120</v>
       </c>
-      <c r="D80" s="26">
+      <c r="D80" s="27">
         <v>60</v>
       </c>
-      <c r="E80" s="26">
+      <c r="E80" s="27">
         <v>0</v>
       </c>
       <c r="F80" s="16">
@@ -21738,10 +22133,10 @@
       <c r="C81" s="16">
         <v>180</v>
       </c>
-      <c r="D81" s="26">
+      <c r="D81" s="27">
         <v>35</v>
       </c>
-      <c r="E81" s="26">
+      <c r="E81" s="27">
         <v>0</v>
       </c>
       <c r="F81" s="16">
@@ -21816,10 +22211,10 @@
       <c r="C82" s="16">
         <v>400</v>
       </c>
-      <c r="D82" s="26">
+      <c r="D82" s="27">
         <v>28</v>
       </c>
-      <c r="E82" s="26">
+      <c r="E82" s="27">
         <v>0</v>
       </c>
       <c r="F82" s="16">
@@ -21894,10 +22289,10 @@
       <c r="C83" s="16">
         <v>1200</v>
       </c>
-      <c r="D83" s="26">
+      <c r="D83" s="27">
         <v>9</v>
       </c>
-      <c r="E83" s="26">
+      <c r="E83" s="27">
         <v>0</v>
       </c>
       <c r="F83" s="16">
@@ -21972,10 +22367,10 @@
       <c r="C84" s="16">
         <v>45</v>
       </c>
-      <c r="D84" s="26">
+      <c r="D84" s="27">
         <v>130</v>
       </c>
-      <c r="E84" s="26">
+      <c r="E84" s="27">
         <v>0</v>
       </c>
       <c r="F84" s="16">
@@ -22050,10 +22445,10 @@
       <c r="C85" s="16">
         <v>25</v>
       </c>
-      <c r="D85" s="26">
+      <c r="D85" s="27">
         <v>400</v>
       </c>
-      <c r="E85" s="26">
+      <c r="E85" s="27">
         <v>0</v>
       </c>
       <c r="F85" s="16">
@@ -22128,10 +22523,10 @@
       <c r="C86" s="16">
         <v>35</v>
       </c>
-      <c r="D86" s="26">
+      <c r="D86" s="27">
         <v>160</v>
       </c>
-      <c r="E86" s="26">
+      <c r="E86" s="27">
         <v>0</v>
       </c>
       <c r="F86" s="16">
@@ -22206,10 +22601,10 @@
       <c r="C87" s="16">
         <v>60</v>
       </c>
-      <c r="D87" s="26">
+      <c r="D87" s="27">
         <v>220</v>
       </c>
-      <c r="E87" s="26">
+      <c r="E87" s="27">
         <v>0</v>
       </c>
       <c r="F87" s="16">
@@ -22284,10 +22679,10 @@
       <c r="C88" s="16">
         <v>150</v>
       </c>
-      <c r="D88" s="26">
+      <c r="D88" s="27">
         <v>70</v>
       </c>
-      <c r="E88" s="26">
+      <c r="E88" s="27">
         <v>0</v>
       </c>
       <c r="F88" s="16">
@@ -22362,10 +22757,10 @@
       <c r="C89" s="16">
         <v>120</v>
       </c>
-      <c r="D89" s="26">
+      <c r="D89" s="27">
         <v>60</v>
       </c>
-      <c r="E89" s="26">
+      <c r="E89" s="27">
         <v>0</v>
       </c>
       <c r="F89" s="16">
@@ -22440,10 +22835,10 @@
       <c r="C90" s="16">
         <v>180</v>
       </c>
-      <c r="D90" s="26">
+      <c r="D90" s="27">
         <v>35</v>
       </c>
-      <c r="E90" s="26">
+      <c r="E90" s="27">
         <v>0</v>
       </c>
       <c r="F90" s="16">
@@ -22518,10 +22913,10 @@
       <c r="C91" s="16">
         <v>400</v>
       </c>
-      <c r="D91" s="26">
+      <c r="D91" s="27">
         <v>28</v>
       </c>
-      <c r="E91" s="26">
+      <c r="E91" s="27">
         <v>0</v>
       </c>
       <c r="F91" s="16">
@@ -22596,10 +22991,10 @@
       <c r="C92" s="16">
         <v>1200</v>
       </c>
-      <c r="D92" s="26">
+      <c r="D92" s="27">
         <v>9</v>
       </c>
-      <c r="E92" s="26">
+      <c r="E92" s="27">
         <v>0</v>
       </c>
       <c r="F92" s="16">
@@ -22674,10 +23069,10 @@
       <c r="C93" s="16">
         <v>45</v>
       </c>
-      <c r="D93" s="26">
+      <c r="D93" s="27">
         <v>130</v>
       </c>
-      <c r="E93" s="26">
+      <c r="E93" s="27">
         <v>0</v>
       </c>
       <c r="F93" s="16">

</xml_diff>

<commit_message>
DOC-003: rediseño editorial del PDF — justificación real por reparto de espacio entre palabras (última línea natural, tope editorial, cruce de páginas justificado, control de huérfanas), paginación por niveles con capítulos en flujo y grupos apaisados sin páginas verticales vacías, tablas corporativas sin rejilla con suelos tipográficos 7,5/7 pt y alineación por contenido; DOCX coherente; guía editorial, informe de densidad, evidencias antes/después y 23 pruebas nuevas (medición posicional, no declarativa)
</commit_message>
<xml_diff>
--- a/docs/ejemplos/Ejemplo_Clinica_Libro_con_formulas.xlsx
+++ b/docs/ejemplos/Ejemplo_Clinica_Libro_con_formulas.xlsx
@@ -801,7 +801,7 @@
         <v>Fecha de exportación:</v>
       </c>
       <c r="B7" s="2" t="str">
-        <v>26/10/2026, 0:40:10</v>
+        <v>26/10/2026, 2:20:44</v>
       </c>
     </row>
     <row r="8">
@@ -12339,7 +12339,7 @@
         <v>FINANCIACION_ANO0</v>
       </c>
       <c r="C4" s="2" t="str">
-        <v>Los gastos de la fase de montaje del año 0 — salidas de caja explícitas no capitalizables y NO incluidas en la inversión total (nómina de montaje 0,8: total 0,8 kUSD) — quedan SIN cobertura temporal: la necesidad total del arranque (inversión 1.480,0 + salidas netas del año 0 = 1.480,8 kUSD) excede las fuentes con desembolso efectivo en el año 0 (1.480,0 kUSD) en 0,8 kUSD. La financiación comprometida total (1.480,0 kUSD) tampoco cubre la necesidad total (1.480,8 kUSD): brecha nominal de 0,8 kUSD. Financie esa brecha (mayor capital de trabajo, aporte anticipado o crédito con desembolso en el año 0) o declárela expresamente como supuesto pendiente. El gasto NO se deduce del resultado contable después de impuestos del año 0.</v>
+        <v>Arranque del año 0 — salidas de caja explícitas no capitalizables y NO incluidas en la inversión total (nómina de montaje 0,8: total 0,8 kUSD) — queda SIN cobertura temporal: la necesidad total del arranque (inversión 1.480,0 + salidas netas del año 0 = 1.480,8 kUSD) excede las fuentes con desembolso efectivo en el año 0 (1.480,0 kUSD) en 0,8 kUSD. La financiación comprometida total (1.480,0 kUSD) tampoco cubre la necesidad total (1.480,8 kUSD): brecha nominal de 0,8 kUSD. Financie esa brecha (mayor capital de trabajo, aporte anticipado o crédito con desembolso en el año 0) o declárela expresamente como supuesto pendiente. El gasto NO se deduce del resultado contable después de impuestos del año 0.</v>
       </c>
       <c r="D4" s="2" t="str">
         <v>financiero</v>

</xml_diff>